<commit_message>
feat: complete v3.5 pre-sales sizing workflow
</commit_message>
<xml_diff>
--- a/docs/examples/si-sizing-example.xlsx
+++ b/docs/examples/si-sizing-example.xlsx
@@ -2,9 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객 요구사항" sheetId="1" r:id="Ra584d3771b414dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구성안 비교" sheetId="2" r:id="R792d886c8db74704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PoC 체크리스트" sheetId="3" r:id="R894791047060418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객 요구사항" sheetId="1" r:id="Rf03aed76ca9f49ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가격·TCO 가정" sheetId="2" r:id="R42ba65b5c2284ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구성안 비교" sheetId="3" r:id="R283696fb477d4b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인프라 BOM" sheetId="4" r:id="R7905410833134fc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PoC 체크리스트" sheetId="5" r:id="R7e47fd6d46244cad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,10 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="#,##0"/>
+  <x:numFmts count="3">
+    <x:numFmt numFmtId="200" formatCode="0%"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0"/>
+    <x:numFmt numFmtId="202" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -33,6 +37,17 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -150,7 +165,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="24">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -162,11 +177,19 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -393,7 +416,7 @@
       <x:c r="A4" s="7" t="str">
         <x:v>프로젝트</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>사내 문서 RAG 구축</x:v>
       </x:c>
     </x:row>
@@ -401,72 +424,142 @@
       <x:c r="A5" s="7" t="str">
         <x:v>구축 목적</x:v>
       </x:c>
-      <x:c r="B5" s="8" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>사내 문서 검색·질의응답</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="str">
-        <x:v>주 모델</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>Qwen 계열 32B</x:v>
+        <x:v>고객 업종</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>제조·일반기업</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7" t="str">
-        <x:v>전체 사용자</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="n">
-        <x:v>100</x:v>
-      </x:c>
+        <x:v>상담 담당자</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7" t="str">
-        <x:v>동시 요청</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="n">
-        <x:v>10</x:v>
+        <x:v>보안</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>내부망·외부 반출 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="str">
-        <x:v>평균 입력 토큰</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="n">
-        <x:v>4096</x:v>
+        <x:v>주 모델</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Qwen 계열 32B</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7" t="str">
-        <x:v>평균 출력 토큰</x:v>
-      </x:c>
-      <x:c r="B10" s="8" t="n">
-        <x:v>500</x:v>
+        <x:v>전체 사용자</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="n">
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="str">
-        <x:v>목표 응답시간</x:v>
-      </x:c>
-      <x:c r="B11" s="8" t="str">
-        <x:v>8초</x:v>
+        <x:v>동시 요청</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="n">
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7" t="str">
+        <x:v>QPS</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="7" t="str">
+        <x:v>평균 입력 토큰</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="n">
+        <x:v>4096</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7" t="str">
+        <x:v>최대 입력 토큰</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="n">
+        <x:v>16384</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="7" t="str">
+        <x:v>평균 출력 토큰</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="n">
+        <x:v>500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="7" t="str">
+        <x:v>TTFT p95</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="7" t="str">
+        <x:v>전체 지연 p95</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="7" t="str">
+        <x:v>일 운영시간</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="7" t="str">
         <x:v>가용성</x:v>
       </x:c>
-      <x:c r="B12" s="8" t="str">
+      <x:c r="B19" s="11" t="str">
         <x:v>HA</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="9" t="str">
+    <x:row r="20">
+      <x:c r="A20" s="7" t="str">
         <x:v>트래픽 증가 여유</x:v>
       </x:c>
-      <x:c r="B13" s="10" t="str">
-        <x:v>30%</x:v>
+      <x:c r="B20" s="13" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="7" t="str">
+        <x:v>벡터 데이터 GB</x:v>
+      </x:c>
+      <x:c r="B21" s="11" t="n">
+        <x:v>500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="9" t="str">
+        <x:v>로그 GB/일</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="n">
+        <x:v>10</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -481,17 +574,173 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>가격·TCO 가정 (파란 글씨 입력)</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="4" t="str">
+        <x:v>항목</x:v>
+      </x:c>
+      <x:c r="B3" s="4" t="str">
+        <x:v>값</x:v>
+      </x:c>
+      <x:c r="C3" s="4" t="str">
+        <x:v>단위</x:v>
+      </x:c>
+      <x:c r="D3" s="4" t="str">
+        <x:v>설명</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>환율</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="n">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>KRW/USD</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>계획 가정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>전력 단가</x:v>
+      </x:c>
+      <x:c r="B5" s="15" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>KRW/kWh</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>고객 계약 단가로 수정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>연 유지보수율</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>구매비 기준</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>RTX 6000 Ada</x:v>
+      </x:c>
+      <x:c r="B7" s="15" t="n">
+        <x:v>8500</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>USD/GPU</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>공급사 견적 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>H100 PCIe</x:v>
+      </x:c>
+      <x:c r="B8" s="15" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>USD/GPU</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>공급사 견적 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>H200 SXM</x:v>
+      </x:c>
+      <x:c r="B9" s="15" t="n">
+        <x:v>40000</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>USD/GPU</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>공급사 견적 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>서버 플랫폼</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="n">
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>USD/server</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>CPU·RAM 기본</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>네트워크·스토리지</x:v>
+      </x:c>
+      <x:c r="B11" s="15" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>USD/server</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>초기 가정</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -508,156 +757,467 @@
       <x:c r="I1" s="2"/>
       <x:c r="J1" s="2"/>
       <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
         <x:v>구성안</x:v>
       </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="B3" s="17" t="str">
         <x:v>GPU</x:v>
       </x:c>
-      <x:c r="C3" s="11" t="str">
+      <x:c r="C3" s="17" t="str">
         <x:v>GPU 수</x:v>
       </x:c>
-      <x:c r="D3" s="11" t="str">
-        <x:v>노드</x:v>
-      </x:c>
-      <x:c r="E3" s="11" t="str">
+      <x:c r="D3" s="17" t="str">
+        <x:v>서버</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="str">
+        <x:v>GPU/서버</x:v>
+      </x:c>
+      <x:c r="F3" s="17" t="str">
         <x:v>CPU 코어</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="str">
+      <x:c r="G3" s="17" t="str">
         <x:v>RAM GB</x:v>
       </x:c>
-      <x:c r="G3" s="11" t="str">
+      <x:c r="H3" s="17" t="str">
         <x:v>NVMe TB</x:v>
       </x:c>
-      <x:c r="H3" s="11" t="str">
+      <x:c r="I3" s="17" t="str">
         <x:v>네트워크</x:v>
       </x:c>
-      <x:c r="I3" s="11" t="str">
+      <x:c r="J3" s="17" t="str">
         <x:v>전력 W</x:v>
       </x:c>
-      <x:c r="J3" s="11" t="str">
+      <x:c r="K3" s="17" t="str">
+        <x:v>장애 잔여</x:v>
+      </x:c>
+      <x:c r="L3" s="17" t="str">
+        <x:v>도입비 KRW</x:v>
+      </x:c>
+      <x:c r="M3" s="17" t="str">
+        <x:v>연 전력비</x:v>
+      </x:c>
+      <x:c r="N3" s="17" t="str">
+        <x:v>3년 TCO</x:v>
+      </x:c>
+      <x:c r="O3" s="6" t="str">
         <x:v>신뢰도</x:v>
-      </x:c>
-      <x:c r="K3" s="6" t="str">
-        <x:v>용도</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
         <x:v>경제형</x:v>
       </x:c>
-      <x:c r="B4" s="12" t="str">
+      <x:c r="B4" s="18" t="str">
         <x:v>RTX 6000 Ada 48GB</x:v>
       </x:c>
-      <x:c r="C4" s="14" t="n">
+      <x:c r="C4" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D4" s="14" t="n">
+      <x:c r="D4" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E4" s="14" t="n">
+      <x:c r="E4" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F4" s="20" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="F4" s="14" t="n">
+      <x:c r="G4" s="20" t="n">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="G4" s="14" t="n">
+      <x:c r="H4" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H4" s="14" t="str">
+      <x:c r="I4" s="20" t="str">
         <x:v>25GbE</x:v>
       </x:c>
-      <x:c r="I4" s="14" t="n">
+      <x:c r="J4" s="20" t="n">
         <x:v>2500</x:v>
       </x:c>
-      <x:c r="J4" s="12" t="str">
+      <x:c r="K4" s="20" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L4" s="22" t="n">
+        <x:f>(C4*'가격·TCO 가정'!$B$7+D4*('가격·TCO 가정'!$B$10+'가격·TCO 가정'!$B$11))*'가격·TCO 가정'!$B$4</x:f>
+        <x:v>56000000</x:v>
+      </x:c>
+      <x:c r="M4" s="22" t="n">
+        <x:f>J4/1000*'고객 요구사항'!$B$18*365*'가격·TCO 가정'!$B$5</x:f>
+        <x:v>3285000</x:v>
+      </x:c>
+      <x:c r="N4" s="22" t="n">
+        <x:f>L4+M4*3+L4*'가격·TCO 가정'!$B$6*3</x:f>
+        <x:v>82655000</x:v>
+      </x:c>
+      <x:c r="O4" s="8" t="str">
         <x:v>낮음</x:v>
-      </x:c>
-      <x:c r="K4" s="8" t="str">
-        <x:v>PoC·제한 운영</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="7" t="str">
         <x:v>권장형</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="str">
+      <x:c r="B5" s="18" t="str">
         <x:v>H100 PCIe 80GB</x:v>
       </x:c>
-      <x:c r="C5" s="14" t="n">
+      <x:c r="C5" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="14" t="n">
+      <x:c r="D5" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E5" s="14" t="n">
+      <x:c r="E5" s="20" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F5" s="20" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="F5" s="14" t="n">
+      <x:c r="G5" s="20" t="n">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="G5" s="14" t="n">
+      <x:c r="H5" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H5" s="14" t="str">
+      <x:c r="I5" s="20" t="str">
         <x:v>100GbE</x:v>
       </x:c>
-      <x:c r="I5" s="14" t="n">
+      <x:c r="J5" s="20" t="n">
         <x:v>3500</x:v>
       </x:c>
-      <x:c r="J5" s="12" t="str">
+      <x:c r="K5" s="20" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L5" s="22" t="n">
+        <x:f>(C5*'가격·TCO 가정'!$B$8+D5*('가격·TCO 가정'!$B$10+'가격·TCO 가정'!$B$11))*'가격·TCO 가정'!$B$4</x:f>
+        <x:v>116200000</x:v>
+      </x:c>
+      <x:c r="M5" s="22" t="n">
+        <x:f>J5/1000*'고객 요구사항'!$B$18*365*'가격·TCO 가정'!$B$5</x:f>
+        <x:v>4599000</x:v>
+      </x:c>
+      <x:c r="N5" s="22" t="n">
+        <x:f>L5+M5*3+L5*'가격·TCO 가정'!$B$6*3</x:f>
+        <x:v>164857000</x:v>
+      </x:c>
+      <x:c r="O5" s="8" t="str">
         <x:v>중간</x:v>
-      </x:c>
-      <x:c r="K5" s="8" t="str">
-        <x:v>운영 권장</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="9" t="str">
         <x:v>확장형</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="str">
+      <x:c r="B6" s="19" t="str">
         <x:v>H200 SXM 141GB</x:v>
       </x:c>
-      <x:c r="C6" s="15" t="n">
+      <x:c r="C6" s="21" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D6" s="15" t="n">
+      <x:c r="D6" s="21" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E6" s="15" t="n">
+      <x:c r="E6" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F6" s="21" t="n">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="F6" s="15" t="n">
+      <x:c r="G6" s="21" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="G6" s="15" t="n">
+      <x:c r="H6" s="21" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H6" s="15" t="str">
-        <x:v>200GbE 검토</x:v>
-      </x:c>
-      <x:c r="I6" s="15" t="n">
+      <x:c r="I6" s="21" t="str">
+        <x:v>200GbE</x:v>
+      </x:c>
+      <x:c r="J6" s="21" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="J6" s="13" t="str">
+      <x:c r="K6" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L6" s="23" t="n">
+        <x:f>(C6*'가격·TCO 가정'!$B$9+D6*('가격·TCO 가정'!$B$10+'가격·TCO 가정'!$B$11))*'가격·TCO 가정'!$B$4</x:f>
+        <x:v>256200000</x:v>
+      </x:c>
+      <x:c r="M6" s="23" t="n">
+        <x:f>J6/1000*'고객 요구사항'!$B$18*365*'가격·TCO 가정'!$B$5</x:f>
+        <x:v>7884000</x:v>
+      </x:c>
+      <x:c r="N6" s="23" t="n">
+        <x:f>L6+M6*3+L6*'가격·TCO 가정'!$B$6*3</x:f>
+        <x:v>356712000</x:v>
+      </x:c>
+      <x:c r="O6" s="10" t="str">
         <x:v>중간</x:v>
-      </x:c>
-      <x:c r="K6" s="10" t="str">
-        <x:v>성장·이중화</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A1:O1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>권장형 인프라 BOM</x:v>
+      </x:c>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="5" t="str">
+        <x:v>구분</x:v>
+      </x:c>
+      <x:c r="B3" s="17" t="str">
+        <x:v>항목</x:v>
+      </x:c>
+      <x:c r="C3" s="17" t="str">
+        <x:v>수량</x:v>
+      </x:c>
+      <x:c r="D3" s="17" t="str">
+        <x:v>요구 조건</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="str">
+        <x:v>검증</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>비고</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="7" t="str">
+        <x:v>GPU</x:v>
+      </x:c>
+      <x:c r="B4" s="18" t="str">
+        <x:v>H100 PCIe 80GB</x:v>
+      </x:c>
+      <x:c r="C4" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D4" s="18" t="str">
+        <x:v>서버당 2</x:v>
+      </x:c>
+      <x:c r="E4" s="18" t="str">
+        <x:v>벤더 견적</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>최종 SKU 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="7" t="str">
+        <x:v>서버</x:v>
+      </x:c>
+      <x:c r="B5" s="18" t="str">
+        <x:v>2U/4U GPU 서버</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="18" t="str">
+        <x:v>PCIe Gen5</x:v>
+      </x:c>
+      <x:c r="E5" s="18" t="str">
+        <x:v>토폴로지</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="str">
+        <x:v>CPU-GPU-NIC 경로</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="7" t="str">
+        <x:v>CPU</x:v>
+      </x:c>
+      <x:c r="B6" s="18" t="str">
+        <x:v>서버 CPU</x:v>
+      </x:c>
+      <x:c r="C6" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" s="18" t="str">
+        <x:v>총 48코어+</x:v>
+      </x:c>
+      <x:c r="E6" s="18" t="str">
+        <x:v>코어/GPU</x:v>
+      </x:c>
+      <x:c r="F6" s="8" t="str">
+        <x:v>NUMA 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="7" t="str">
+        <x:v>RAM</x:v>
+      </x:c>
+      <x:c r="B7" s="18" t="str">
+        <x:v>ECC RAM</x:v>
+      </x:c>
+      <x:c r="C7" s="18" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D7" s="18" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="E7" s="18" t="str">
+        <x:v>용량</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="str">
+        <x:v>모델·캐시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="7" t="str">
+        <x:v>스토리지</x:v>
+      </x:c>
+      <x:c r="B8" s="18" t="str">
+        <x:v>NVMe</x:v>
+      </x:c>
+      <x:c r="C8" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D8" s="18" t="str">
+        <x:v>TB+</x:v>
+      </x:c>
+      <x:c r="E8" s="18" t="str">
+        <x:v>처리량</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="str">
+        <x:v>모델·벡터DB·로그</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="7" t="str">
+        <x:v>네트워크</x:v>
+      </x:c>
+      <x:c r="B9" s="18" t="str">
+        <x:v>100GbE NIC</x:v>
+      </x:c>
+      <x:c r="C9" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D9" s="18" t="str">
+        <x:v>이중화</x:v>
+      </x:c>
+      <x:c r="E9" s="18" t="str">
+        <x:v>스위치</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="str">
+        <x:v>East-West</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="7" t="str">
+        <x:v>패브릭</x:v>
+      </x:c>
+      <x:c r="B10" s="18" t="str">
+        <x:v>Ethernet/InfiniBand</x:v>
+      </x:c>
+      <x:c r="C10" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="18" t="str">
+        <x:v>설계 선택</x:v>
+      </x:c>
+      <x:c r="E10" s="18" t="str">
+        <x:v>지연</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="str">
+        <x:v>멀티노드 시 검토</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="7" t="str">
+        <x:v>전력</x:v>
+      </x:c>
+      <x:c r="B11" s="18" t="str">
+        <x:v>랙 전력</x:v>
+      </x:c>
+      <x:c r="C11" s="18" t="n">
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="D11" s="18" t="str">
+        <x:v>W+</x:v>
+      </x:c>
+      <x:c r="E11" s="18" t="str">
+        <x:v>PDU</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>피크 여유</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="7" t="str">
+        <x:v>UPS</x:v>
+      </x:c>
+      <x:c r="B12" s="18" t="str">
+        <x:v>UPS</x:v>
+      </x:c>
+      <x:c r="C12" s="18" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D12" s="18" t="str">
+        <x:v>분</x:v>
+      </x:c>
+      <x:c r="E12" s="18" t="str">
+        <x:v>시설</x:v>
+      </x:c>
+      <x:c r="F12" s="8" t="str">
+        <x:v>정전 정책</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="9" t="str">
+        <x:v>운영</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>백업·모니터링</x:v>
+      </x:c>
+      <x:c r="C13" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D13" s="19" t="str">
+        <x:v>일 백업·GPU/p95/오류</x:v>
+      </x:c>
+      <x:c r="E13" s="19" t="str">
+        <x:v>PoC</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="str">
+        <x:v>감사로그 선택</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -679,10 +1239,10 @@
       <x:c r="A3" s="5" t="str">
         <x:v>상태</x:v>
       </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="B3" s="17" t="str">
         <x:v>검증 항목</x:v>
       </x:c>
-      <x:c r="C3" s="11" t="str">
+      <x:c r="C3" s="17" t="str">
         <x:v>합격 기준</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
@@ -693,10 +1253,10 @@
       <x:c r="A4" s="7" t="str">
         <x:v>미착수</x:v>
       </x:c>
-      <x:c r="B4" s="12" t="str">
+      <x:c r="B4" s="18" t="str">
         <x:v>모델 버전·양자화·런타임 확정</x:v>
       </x:c>
-      <x:c r="C4" s="12" t="str">
+      <x:c r="C4" s="18" t="str">
         <x:v>배포 대상과 동일</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str"/>
@@ -705,10 +1265,10 @@
       <x:c r="A5" s="7" t="str">
         <x:v>미착수</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="str">
+      <x:c r="B5" s="18" t="str">
         <x:v>TTFT 측정</x:v>
       </x:c>
-      <x:c r="C5" s="12" t="str">
+      <x:c r="C5" s="18" t="str">
         <x:v>2초 이내</x:v>
       </x:c>
       <x:c r="D5" s="8" t="str">
@@ -719,10 +1279,10 @@
       <x:c r="A6" s="7" t="str">
         <x:v>미착수</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="str">
+      <x:c r="B6" s="18" t="str">
         <x:v>생성 속도</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="str">
+      <x:c r="C6" s="18" t="str">
         <x:v>목표 tokens/s 충족</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
@@ -733,10 +1293,10 @@
       <x:c r="A7" s="7" t="str">
         <x:v>미착수</x:v>
       </x:c>
-      <x:c r="B7" s="12" t="str">
+      <x:c r="B7" s="18" t="str">
         <x:v>동시 요청 부하</x:v>
       </x:c>
-      <x:c r="C7" s="12" t="str">
+      <x:c r="C7" s="18" t="str">
         <x:v>10명·오류율 1% 미만</x:v>
       </x:c>
       <x:c r="D7" s="8" t="str">
@@ -747,10 +1307,10 @@
       <x:c r="A8" s="7" t="str">
         <x:v>미착수</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="str">
+      <x:c r="B8" s="18" t="str">
         <x:v>장애 전환</x:v>
       </x:c>
-      <x:c r="C8" s="12" t="str">
+      <x:c r="C8" s="18" t="str">
         <x:v>서비스 목표 충족</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
@@ -761,10 +1321,10 @@
       <x:c r="A9" s="7" t="str">
         <x:v>미착수</x:v>
       </x:c>
-      <x:c r="B9" s="12" t="str">
+      <x:c r="B9" s="18" t="str">
         <x:v>모니터링</x:v>
       </x:c>
-      <x:c r="C9" s="12" t="str">
+      <x:c r="C9" s="18" t="str">
         <x:v>GPU·지연·오류 수집</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str"/>
@@ -773,10 +1333,10 @@
       <x:c r="A10" s="9" t="str">
         <x:v>주의</x:v>
       </x:c>
-      <x:c r="B10" s="13" t="str">
+      <x:c r="B10" s="19" t="str">
         <x:v>최종 수량</x:v>
       </x:c>
-      <x:c r="C10" s="13" t="str">
+      <x:c r="C10" s="19" t="str">
         <x:v>실제 PoC 후 확정</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">

</xml_diff>